<commit_message>
Limit plan comparison download to medical (health) plans only
Drop Dental / Vision / Supplemental from the generated Excel + PDF so
the download is the 15 health plans only. The Dental/Vision/Supplemental
data still parses for the count validation but is no longer exported.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JafzPN5ofrARY5Fev86pBG
</commit_message>
<xml_diff>
--- a/client/public/downloads/Kennion-Health-Plans-Comparison.xlsx
+++ b/client/public/downloads/Kennion-Health-Plans-Comparison.xlsx
@@ -8,10 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Medical" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dental" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Vision" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Voluntary Benefits" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Voluntary Hospital" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -132,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -175,12 +171,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2000,980 +1990,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Kennion Health Plans — Dental Comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>All plans include: 24/7 virtual care, concierge support, and a Visa card to help pay for care.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Benefit</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Advantage Dental (w/ Ortho)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Complete Dental (w/ Ortho)</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Value Dental (w/ Ortho)</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Complete Dental</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Value Dental</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Basic Dental</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Choice Dental</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Deductible</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>$25</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>$50</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>$50</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>$50</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>$50</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>$50</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>$50</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Annual Maximum Benefit</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>$2,500</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>$1,500</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>$1,000</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>$1,500</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>$1,000</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>$750</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>$750</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Lifetime Ortho Maximum</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>$2,500</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>$1,500</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>$1,000</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>COVERED SERVICES</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Preventative (Plan Pays)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Basic (Plan Pays)</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Major (Plan Pays)</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Ortho (Plan Pays)</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>50%</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Benefit descriptions only — not a contract. Rates are quoted separately and subject to final underwriting. Questions? Hunter Shepherd (hunter@kennion.com).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Kennion Health Plans — Vision Comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>All plans include: 24/7 virtual care, concierge support, and a Visa card to help pay for care.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Benefit</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Premium Vision</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Standard Vision</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Value Vision</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Base Vision</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Exam Copayment</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>$10</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>$20</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Material Copayment</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>$20</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>$20</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Exam Every</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>12 Months</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>12 Months</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>12 Months</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>12 Months</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Lenses Every</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>12 Months</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>12 Months</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>12 Months</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>24 Months</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Frames Every</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>12 Months</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>24 Months</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>24 Months</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>24 Months</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>ALLOWANCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Frames</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>$180 / $200</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>$150 / $170</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>$150 / $170</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>$130 / $150</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Elective Contact Lenses</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>$180</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>$130</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>$150</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Necessary Contact Lenses</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Covered after copay</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Covered after copay</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Covered after copay</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Covered after copay</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Benefit descriptions only — not a contract. Rates are quoted separately and subject to final underwriting. Questions? Hunter Shepherd (hunter@kennion.com).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A10:E10"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Kennion Health Plans — Voluntary Benefits</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Benefit</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Coverage</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>Voluntary Life / AD&amp;D</t>
-        </is>
-      </c>
-      <c r="B4" s="17" t="inlineStr">
-        <is>
-          <t>$100,000 Employee / $50,000 Spouse / $10,000 Child(ren)
-(Rates based on age.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Voluntary Short-Term Disability</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>$500 weekly benefit
-(Employee only. Rates based on age.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Voluntary Accident</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Fixed-indemnity accident benefits for covered injuries.
-(Composite rates — see Supplemental in your quote.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Voluntary Cancer</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Fixed-indemnity cancer benefits including diagnosis and treatment.
-(Composite rates — see Supplemental in your quote.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>Voluntary Critical Illness</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>$10,000 Employee / $5,000 Spouse / $2,500 Child(ren)
-(Rates based on age.)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Kennion Health Plans — Voluntary Hospital Comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>All plans include: 24/7 virtual care, concierge support, and a Visa card to help pay for care.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Benefit</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Choice Plan</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Basic Plan</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Preferred Plan</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Enhanced Plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>INPATIENT HOSPITAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Hospital Admission</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>$500 + $200 / day</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>$1,000 + $250 / day</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>$2,000 + $300 / day</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>$3,000 + $400 / day</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>OTHER FACILITY BENEFITS</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Emergency Room / Urgent Care Facility</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>$200 ER / $50 Urgent Care</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>$300 ER / $75 Urgent Care</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>$400 ER / $100 Urgent Care</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>$500 ER / $150 Urgent Care</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>SURGERIES</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Inpatient / Outpatient Surgery</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Up to $500</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Up to $1,000</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Up to $1,500</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Up to $2,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>Benefit descriptions only — not a contract. Rates are quoted separately and subject to final underwriting. Questions? Hunter Shepherd (hunter@kennion.com).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A9:E9"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>